<commit_message>
feat: Enhance Reflections export with auto-sizing, event handling, and user guidance; update download template link
</commit_message>
<xml_diff>
--- a/public/download/Template_Import_Refleksi.xlsx
+++ b/public/download/Template_Import_Refleksi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zacky\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A46C0F-2967-47E6-9C54-4D1E7B5301B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A8D7DA-FA8A-4AF5-AD99-D967F7611EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5112" yWindow="2712" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template Import Refleksi" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t>Jenis Penilaian</t>
   </si>
@@ -51,101 +51,137 @@
     <t>Kelas</t>
   </si>
   <si>
+    <t>PETUNJUK PENGISIAN (KOLOM INI TIDAK AKAN DIIMPORT):</t>
+  </si>
+  <si>
+    <t>1. Kategori Predikat yang diizinkan (Wajib sama persis):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Sangat Baik (Untuk Nilai 91-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Baik (Untuk Nilai 76-90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Cukup (Untuk Nilai 61-75)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Perlu Bimbingan (Untuk Nilai &lt;60)</t>
+  </si>
+  <si>
+    <t>2. Jenis Penilaian hanya ada dua:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Kinerja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Proyek</t>
+  </si>
+  <si>
+    <t>3. Cara mengisi lebih dari satu poin refleksi:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Gunakan Enter (Alt+Enter di dalam Excel) ATAU karakter titik koma (;) untuk memisahkan antar poin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Contoh format sel: Anak sangat aktif; Berani tampil ke depan</t>
+  </si>
+  <si>
+    <t>Menunjukkan usaha awal dalam memahami langkah proyek dengan arahan guru.</t>
+  </si>
+  <si>
+    <t>Perlu meningkatkan perencanaan, pengumpulan data, dan penyajian hasil agar lebih terarah.</t>
+  </si>
+  <si>
+    <t>Diberi bimbingan tambahan dan contoh proyek sederhana untuk memperkuat pemahaman dasar.</t>
+  </si>
+  <si>
+    <t>Sudah dapat mengikuti alur pengerjaan proyek dengan arahan minimal.</t>
+  </si>
+  <si>
+    <t>Perlu memperdalam isi dan meningkatkan kerapian penyusunan laporan proyek.</t>
+  </si>
+  <si>
+    <t>Diberi latihan pengayaan melalui proyek lanjutan yang serupa dengan tingkat kesulitan sedikit lebih tinggi.</t>
+  </si>
+  <si>
+    <t>Mampu melaksanakan proyek dengan mandiri dan memahami setiap tahapan secara runtut.</t>
+  </si>
+  <si>
+    <t>Dapat meningkatkan kreativitas dan kemampuan refleksi terhadap hasil proyek.</t>
+  </si>
+  <si>
+    <t>Diberi kesempatan melakukan proyek pengembangan atau proyek lintas tema untuk memperluas wawasan.</t>
+  </si>
+  <si>
+    <t>Menunjukkan kemandirian, kreativitas, dan tanggung jawab tinggi dalam seluruh tahapan proyek.</t>
+  </si>
+  <si>
+    <t>Perlu terus mengembangkan ide orisinal dan memperdalam analisis hasil.</t>
+  </si>
+  <si>
+    <t>Didorong menjadi inspirator atau mentor kecil bagi teman dalam kegiatan proyek berikutnya.</t>
+  </si>
+  <si>
+    <t>Berusaha melaksanakan tugas kinerja meski masih perlu banyak arahan.</t>
+  </si>
+  <si>
+    <t>Perlu meningkatkan ketelitian, koordinasi gerak, dan pemahaman prosedur kerja.</t>
+  </si>
+  <si>
+    <t>Diberi latihan terbimbing dengan contoh langkah kerja sederhana dan pendampingan intensif.</t>
+  </si>
+  <si>
+    <t>Sudah mampu melaksanakan tugas dengan arahan terbatas dan menunjukkan kemauan belajar.</t>
+  </si>
+  <si>
+    <t>Perlu memperbaiki kecepatan dan kerapian dalam melakukan langkah-langkah kinerja.</t>
+  </si>
+  <si>
+    <t>Diberi tugas latihan berulang untuk memperkuat keterampilan dasar dan meningkatkan kepercayaan diri.</t>
+  </si>
+  <si>
+    <t>Melaksanakan tugas kinerja dengan mandiri, teliti, dan sesuai prosedur.</t>
+  </si>
+  <si>
+    <t>Dapat meningkatkan efisiensi waktu dan ketepatan hasil kerja agar lebih optimal.</t>
+  </si>
+  <si>
+    <t>Diberi tantangan kinerja lanjutan dengan variasi situasi agar kemampuan lebih terasah.</t>
+  </si>
+  <si>
+    <t>Menampilkan performa yang sangat baik, kreatif, dan konsisten dalam setiap pelaksanaan tugas.</t>
+  </si>
+  <si>
+    <t>Perlu terus mempertahankan performa serta menularkan semangat kerja kepada rekan lain.</t>
+  </si>
+  <si>
+    <t>Dilibatkan dalam demonstrasi atau penugasan lanjutan sebagai model praktik baik.</t>
+  </si>
+  <si>
     <t>proyek</t>
   </si>
   <si>
+    <t>kinerja</t>
+  </si>
+  <si>
     <t>Perlu Bimbingan</t>
   </si>
   <si>
-    <t>Menunjukkan usaha awal dalam memahami langkah proyek dengan arahan guru.</t>
-  </si>
-  <si>
-    <t>Perlu meningkatkan perencanaan, pengumpulan data, dan penyajian hasil agar lebih terarah.</t>
-  </si>
-  <si>
-    <t>Diberi bimbingan tambahan dan contoh proyek sederhana untuk memperkuat pemahaman dasar.</t>
-  </si>
-  <si>
     <t>Cukup</t>
   </si>
   <si>
-    <t>Sudah dapat mengikuti alur pengerjaan proyek dengan arahan minimal.</t>
-  </si>
-  <si>
-    <t>Perlu memperdalam isi dan meningkatkan kerapian penyusunan laporan proyek.</t>
-  </si>
-  <si>
-    <t>Diberi latihan pengayaan melalui proyek lanjutan yang serupa dengan tingkat kesulitan sedikit lebih tinggi.</t>
-  </si>
-  <si>
     <t>Baik</t>
   </si>
   <si>
-    <t>Mampu melaksanakan proyek dengan mandiri dan memahami setiap tahapan secara runtut.</t>
-  </si>
-  <si>
-    <t>Dapat meningkatkan kreativitas dan kemampuan refleksi terhadap hasil proyek.</t>
-  </si>
-  <si>
-    <t>Diberi kesempatan melakukan proyek pengembangan atau proyek lintas tema untuk memperluas wawasan.</t>
-  </si>
-  <si>
     <t>Sangat Baik</t>
-  </si>
-  <si>
-    <t>Menunjukkan kemandirian, kreativitas, dan tanggung jawab tinggi dalam seluruh tahapan proyek.</t>
-  </si>
-  <si>
-    <t>Perlu terus mengembangkan ide orisinal dan memperdalam analisis hasil.</t>
-  </si>
-  <si>
-    <t>Didorong menjadi inspirator atau mentor kecil bagi teman dalam kegiatan proyek berikutnya.</t>
-  </si>
-  <si>
-    <t>Berusaha melaksanakan tugas kinerja meski masih perlu banyak arahan.</t>
-  </si>
-  <si>
-    <t>Perlu meningkatkan ketelitian, koordinasi gerak, dan pemahaman prosedur kerja.</t>
-  </si>
-  <si>
-    <t>Diberi latihan terbimbing dengan contoh langkah kerja sederhana dan pendampingan intensif.</t>
-  </si>
-  <si>
-    <t>Sudah mampu melaksanakan tugas dengan arahan terbatas dan menunjukkan kemauan belajar.</t>
-  </si>
-  <si>
-    <t>Perlu memperbaiki kecepatan dan kerapian dalam melakukan langkah-langkah kinerja.</t>
-  </si>
-  <si>
-    <t>Diberi tugas latihan berulang untuk memperkuat keterampilan dasar dan meningkatkan kepercayaan diri.</t>
-  </si>
-  <si>
-    <t>Melaksanakan tugas kinerja dengan mandiri, teliti, dan sesuai prosedur.</t>
-  </si>
-  <si>
-    <t>Dapat meningkatkan efisiensi waktu dan ketepatan hasil kerja agar lebih optimal.</t>
-  </si>
-  <si>
-    <t>Diberi tantangan kinerja lanjutan dengan variasi situasi agar kemampuan lebih terasah.</t>
-  </si>
-  <si>
-    <t>Menampilkan performa yang sangat baik, kreatif, dan konsisten dalam setiap pelaksanaan tugas.</t>
-  </si>
-  <si>
-    <t>Perlu terus mempertahankan performa serta menularkan semangat kerja kepada rekan lain.</t>
-  </si>
-  <si>
-    <t>Dilibatkan dalam demonstrasi atau penugasan lanjutan sebagai model praktik baik.</t>
-  </si>
-  <si>
-    <t>kinerja</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -158,28 +194,53 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="12"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -187,19 +248,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -505,18 +585,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -536,149 +616,191 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:8" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="4" spans="1:8" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
+    </row>
+    <row r="6" spans="1:8" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    </row>
+    <row r="7" spans="1:8" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
+    </row>
+    <row r="8" spans="1:8" ht="63" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="4" t="s">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="4" t="s">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4" t="s">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="4" t="s">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>